<commit_message>
Update v18.51: Forced Province from DB in app, fixed Excel coordinate recovery, and synced files
</commit_message>
<xml_diff>
--- a/Pipistrelli 2022.xlsx
+++ b/Pipistrelli 2022.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,9 +48,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -493,7 +493,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>44750</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -506,7 +506,6 @@
           <t>Pipistrellus sp.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Viale Margherita, 35</t>
@@ -546,10 +545,9 @@
           <t>morto</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>44745</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -562,7 +560,6 @@
           <t>Pipistrellus sp.</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Via Brescia</t>
@@ -602,10 +599,9 @@
           <t>liberato</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>44754</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -618,7 +614,6 @@
           <t>Pipistrellus sp.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Via San Giorgio</t>
@@ -658,10 +653,9 @@
           <t>morto</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>44746</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -718,10 +712,9 @@
           <t>morto</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>44747</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -778,10 +771,9 @@
           <t>liberato</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>44858</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -794,7 +786,6 @@
           <t>Pipistrellus sp.</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Via Porto</t>
@@ -834,7 +825,6 @@
           <t>morto</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>